<commit_message>
Update Excel catalog for warehouse dimensions and density
</commit_message>
<xml_diff>
--- a/public/data/DS_kho_than_va_ty_khoi.xlsx
+++ b/public/data/DS_kho_than_va_ty_khoi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TTCO_TonKho_App_Repo\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DE7A5BA-906D-4AF3-9601-9832AE739052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35283C7-2E4F-45A1-ADFE-0B6CB5756B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -594,7 +594,7 @@
         <v>48.3</v>
       </c>
       <c r="D2" s="2">
-        <v>36.5</v>
+        <v>1</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>

</xml_diff>